<commit_message>
update : UI 화면 크기 수정
</commit_message>
<xml_diff>
--- a/data/menu.xlsx
+++ b/data/menu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/barkjungha/Desktop/newdev/beginnersClass/class-list/menupan/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80A4AA58-064D-1C4E-BAC6-3032AA727382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B43F194-710D-3F4B-BD96-113918CEE6F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25600" yWindow="600" windowWidth="25600" windowHeight="28200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25600" yWindow="600" windowWidth="25600" windowHeight="28200" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="커피" sheetId="1" r:id="rId1"/>
@@ -169,9 +169,6 @@
     <t>테마</t>
   </si>
   <si>
-    <t>deep-green</t>
-  </si>
-  <si>
     <t>디바이스</t>
   </si>
   <si>
@@ -185,6 +182,10 @@
   </si>
   <si>
     <t>자동전환초</t>
+  </si>
+  <si>
+    <t>cream</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -940,28 +941,28 @@
         <v>47</v>
       </c>
       <c r="B3" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" t="s">
         <v>49</v>
-      </c>
-      <c r="B4" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" t="s">
         <v>51</v>
-      </c>
-      <c r="B5" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -971,7 +972,7 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:B6" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:B2 A4:B6 A3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>